<commit_message>
Venue tracking: Osero (3006 re-route, Li.Fi 3900) + Skybase (1inch 1020) (#19)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hypersync-results/dr_comparison_hypersync.xlsx
+++ b/hypersync-results/dr_comparison_hypersync.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -642,13 +642,13 @@
         <v>1390891.07</v>
       </c>
       <c r="H5" t="n">
-        <v>534444.27</v>
+        <v>534443.5</v>
       </c>
       <c r="I5" t="n">
-        <v>279380.54</v>
+        <v>279379.88</v>
       </c>
       <c r="J5" t="n">
-        <v>9455567.460000001</v>
+        <v>9455566.029999999</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -2288,7 +2288,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3006</t>
         </is>
       </c>
       <c r="B51" t="inlineStr"/>
@@ -2297,16 +2297,18 @@
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+      <c r="H51" t="n">
+        <v>0.77</v>
+      </c>
       <c r="I51" t="n">
-        <v>21.19</v>
+        <v>0.66</v>
       </c>
       <c r="J51" t="n">
-        <v>21.19</v>
+        <v>1.43</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>sUSDS</t>
+          <t>sUSDC, sUSDS</t>
         </is>
       </c>
       <c r="L51" t="inlineStr"/>
@@ -2314,35 +2316,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>3333</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="C52" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="D52" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="E52" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="F52" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="G52" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="H52" t="n">
-        <v>0.24</v>
-      </c>
+          <t>3009</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="n">
-        <v>0.14</v>
+        <v>21.19</v>
       </c>
       <c r="J52" t="n">
-        <v>3.35</v>
+        <v>21.19</v>
       </c>
       <c r="K52" t="inlineStr">
         <is>
@@ -2354,225 +2342,221 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>3333</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>28500.23</v>
+        <v>0.71</v>
       </c>
       <c r="C53" t="n">
-        <v>25181.36</v>
+        <v>0.41</v>
       </c>
       <c r="D53" t="n">
-        <v>29061.49</v>
+        <v>0.48</v>
       </c>
       <c r="E53" t="n">
-        <v>23261.27</v>
+        <v>0.49</v>
       </c>
       <c r="F53" t="n">
-        <v>22648.4</v>
+        <v>0.48</v>
       </c>
       <c r="G53" t="n">
-        <v>19688.27</v>
+        <v>0.39</v>
       </c>
       <c r="H53" t="n">
-        <v>4107.61</v>
+        <v>0.24</v>
       </c>
       <c r="I53" t="n">
-        <v>1523.19</v>
+        <v>0.14</v>
       </c>
       <c r="J53" t="n">
-        <v>153971.83</v>
+        <v>3.35</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>USDS</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
-        </is>
-      </c>
+          <t>sUSDS</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>4011</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
+          <t>4001</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>28500.23</v>
+      </c>
+      <c r="C54" t="n">
+        <v>25181.36</v>
+      </c>
+      <c r="D54" t="n">
+        <v>29061.49</v>
+      </c>
+      <c r="E54" t="n">
+        <v>23261.27</v>
+      </c>
       <c r="F54" t="n">
-        <v>76.34</v>
-      </c>
-      <c r="G54" t="inlineStr"/>
+        <v>22648.4</v>
+      </c>
+      <c r="G54" t="n">
+        <v>19688.27</v>
+      </c>
       <c r="H54" t="n">
-        <v>119.5</v>
+        <v>4107.61</v>
       </c>
       <c r="I54" t="n">
-        <v>7.72</v>
+        <v>1523.19</v>
       </c>
       <c r="J54" t="n">
-        <v>203.56</v>
+        <v>153971.83</v>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>sUSDS</t>
+          <t>USDS</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
+          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>9001</t>
-        </is>
-      </c>
-      <c r="B55" t="n">
-        <v>17730.23</v>
-      </c>
-      <c r="C55" t="n">
-        <v>14347.44</v>
-      </c>
-      <c r="D55" t="n">
-        <v>19582.45</v>
-      </c>
-      <c r="E55" t="n">
-        <v>15967.76</v>
-      </c>
+          <t>4011</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
       <c r="F55" t="n">
-        <v>9527.389999999999</v>
-      </c>
-      <c r="G55" t="n">
-        <v>5835.14</v>
-      </c>
+        <v>76.34</v>
+      </c>
+      <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
-        <v>2750.87</v>
+        <v>119.5</v>
       </c>
       <c r="I55" t="n">
-        <v>1993.6</v>
+        <v>7.72</v>
       </c>
       <c r="J55" t="n">
-        <v>87734.86</v>
+        <v>203.56</v>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>USDS</t>
+          <t>sUSDS</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>9998</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
+          <t>9001</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>17730.23</v>
+      </c>
+      <c r="C56" t="n">
+        <v>14347.44</v>
+      </c>
+      <c r="D56" t="n">
+        <v>19582.45</v>
+      </c>
+      <c r="E56" t="n">
+        <v>15967.76</v>
+      </c>
+      <c r="F56" t="n">
+        <v>9527.389999999999</v>
+      </c>
+      <c r="G56" t="n">
+        <v>5835.14</v>
+      </c>
+      <c r="H56" t="n">
+        <v>2750.87</v>
+      </c>
+      <c r="I56" t="n">
+        <v>1993.6</v>
+      </c>
       <c r="J56" t="n">
-        <v>0.01</v>
+        <v>87734.86</v>
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>sUSDS</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr"/>
+          <t>USDS</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>373.74</v>
-      </c>
-      <c r="C57" t="n">
-        <v>547.46</v>
-      </c>
-      <c r="D57" t="n">
-        <v>1161.68</v>
-      </c>
-      <c r="E57" t="n">
-        <v>1570.26</v>
-      </c>
-      <c r="F57" t="n">
-        <v>1039.27</v>
-      </c>
-      <c r="G57" t="n">
-        <v>734.97</v>
-      </c>
-      <c r="H57" t="n">
-        <v>419.53</v>
-      </c>
-      <c r="I57" t="n">
-        <v>179.36</v>
-      </c>
+          <t>9998</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
+      <c r="C57" t="inlineStr"/>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
       <c r="J57" t="n">
-        <v>6026.26</v>
+        <v>0.01</v>
       </c>
       <c r="K57" t="inlineStr">
         <is>
           <t>sUSDS</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
-        </is>
-      </c>
+      <c r="L57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>77410.08</v>
+        <v>373.74</v>
       </c>
       <c r="C58" t="n">
-        <v>64106.05</v>
+        <v>547.46</v>
       </c>
       <c r="D58" t="n">
-        <v>68681.05</v>
+        <v>1161.68</v>
       </c>
       <c r="E58" t="n">
-        <v>62968.01</v>
+        <v>1570.26</v>
       </c>
       <c r="F58" t="n">
-        <v>59304.61</v>
+        <v>1039.27</v>
       </c>
       <c r="G58" t="n">
-        <v>56940.63</v>
+        <v>734.97</v>
       </c>
       <c r="H58" t="n">
-        <v>36971.31</v>
+        <v>419.53</v>
       </c>
       <c r="I58" t="n">
-        <v>35115.46</v>
+        <v>179.36</v>
       </c>
       <c r="J58" t="n">
-        <v>461497.2</v>
+        <v>6026.26</v>
       </c>
       <c r="K58" t="inlineStr">
         <is>
@@ -2581,49 +2565,93 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
+          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>77410.08</v>
+      </c>
+      <c r="C59" t="n">
+        <v>64106.05</v>
+      </c>
+      <c r="D59" t="n">
+        <v>68681.05</v>
+      </c>
+      <c r="E59" t="n">
+        <v>62968.01</v>
+      </c>
+      <c r="F59" t="n">
+        <v>59304.61</v>
+      </c>
+      <c r="G59" t="n">
+        <v>56940.63</v>
+      </c>
+      <c r="H59" t="n">
+        <v>36971.31</v>
+      </c>
+      <c r="I59" t="n">
+        <v>35115.46</v>
+      </c>
+      <c r="J59" t="n">
+        <v>461497.2</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>sUSDS</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>13425</t>
         </is>
       </c>
-      <c r="B59" t="n">
+      <c r="B60" t="n">
         <v>858.01</v>
       </c>
-      <c r="C59" t="n">
+      <c r="C60" t="n">
         <v>774.97</v>
       </c>
-      <c r="D59" t="n">
+      <c r="D60" t="n">
         <v>858.01</v>
       </c>
-      <c r="E59" t="n">
+      <c r="E60" t="n">
         <v>641.16</v>
       </c>
-      <c r="F59" t="n">
+      <c r="F60" t="n">
         <v>9.67</v>
       </c>
-      <c r="G59" t="n">
+      <c r="G60" t="n">
         <v>9.359999999999999</v>
       </c>
-      <c r="H59" t="n">
+      <c r="H60" t="n">
         <v>5.37</v>
       </c>
-      <c r="I59" t="n">
+      <c r="I60" t="n">
         <v>3.87</v>
       </c>
-      <c r="J59" t="n">
+      <c r="J60" t="n">
         <v>3160.42</v>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="K60" t="inlineStr">
         <is>
           <t>USDS-SKY, sUSDS</t>
         </is>
       </c>
-      <c r="L59" t="inlineStr"/>
+      <c r="L60" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2636,7 +2664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:I83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4748,7 +4776,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>3007</t>
+          <t>3006</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4779,7 +4807,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>3007</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4810,7 +4838,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4841,7 +4869,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4872,12 +4900,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>3333</t>
+          <t>3123</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -4890,60 +4918,56 @@
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G71" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="H71" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>3333</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>soter only</t>
+          <t>both</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>28500.23</v>
+        <v>0</v>
       </c>
       <c r="D72" t="n">
-        <v>25181.36</v>
+        <v>0</v>
       </c>
       <c r="E72" t="n">
-        <v>29061.49</v>
+        <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>23261.27</v>
+        <v>-0</v>
       </c>
       <c r="G72" t="n">
-        <v>22648.4</v>
+        <v>-0.01</v>
       </c>
       <c r="H72" t="n">
-        <v>128652.75</v>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
-        </is>
-      </c>
+        <v>-0.01</v>
+      </c>
+      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>4011</t>
+          <t>3900</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -4959,21 +4983,17 @@
         <v>0</v>
       </c>
       <c r="G73" t="n">
-        <v>76.33</v>
+        <v>0</v>
       </c>
       <c r="H73" t="n">
-        <v>76.33</v>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>4012</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4982,69 +5002,73 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>28500.23</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>25181.36</v>
       </c>
       <c r="E74" t="n">
-        <v>0</v>
+        <v>29061.49</v>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
+        <v>23261.27</v>
       </c>
       <c r="G74" t="n">
-        <v>0</v>
+        <v>22648.4</v>
       </c>
       <c r="H74" t="n">
-        <v>0</v>
-      </c>
-      <c r="I74" t="inlineStr"/>
+        <v>128652.75</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>9001</t>
+          <t>4011</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>soter only</t>
+          <t>both</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>17730.23</v>
+        <v>0</v>
       </c>
       <c r="D75" t="n">
-        <v>14347.44</v>
+        <v>0</v>
       </c>
       <c r="E75" t="n">
-        <v>19582.45</v>
+        <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>15967.76</v>
+        <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>9527.389999999999</v>
+        <v>76.33</v>
       </c>
       <c r="H75" t="n">
-        <v>77155.27</v>
+        <v>76.33</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>9998</t>
+          <t>4012</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -5070,7 +5094,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>9001</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -5079,156 +5103,222 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>373.74</v>
+        <v>17730.23</v>
       </c>
       <c r="D77" t="n">
-        <v>547.46</v>
+        <v>14347.44</v>
       </c>
       <c r="E77" t="n">
-        <v>1161.68</v>
+        <v>19582.45</v>
       </c>
       <c r="F77" t="n">
-        <v>1570.26</v>
+        <v>15967.76</v>
       </c>
       <c r="G77" t="n">
-        <v>1039.27</v>
+        <v>9527.389999999999</v>
       </c>
       <c r="H77" t="n">
-        <v>4692.41</v>
+        <v>77155.27</v>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>9998</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>soter only</t>
+          <t>both</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>77410.08</v>
+        <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>64106.05</v>
+        <v>0</v>
       </c>
       <c r="E78" t="n">
-        <v>68681.05</v>
+        <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>62968.01</v>
+        <v>0</v>
       </c>
       <c r="G78" t="n">
-        <v>59304.61</v>
+        <v>0</v>
       </c>
       <c r="H78" t="n">
-        <v>332469.8</v>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>13425</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>-1.02</v>
+        <v>373.74</v>
       </c>
       <c r="D79" t="n">
-        <v>-0.93</v>
+        <v>547.46</v>
       </c>
       <c r="E79" t="n">
-        <v>-1.02</v>
+        <v>1161.68</v>
       </c>
       <c r="F79" t="n">
-        <v>-0.77</v>
+        <v>1570.26</v>
       </c>
       <c r="G79" t="n">
-        <v>-0.01</v>
+        <v>1039.27</v>
       </c>
       <c r="H79" t="n">
-        <v>-3.75</v>
-      </c>
-      <c r="I79" t="inlineStr"/>
+        <v>4692.41</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>123623963915635</t>
+          <t>10001</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ba only</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>0</v>
+        <v>77410.08</v>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
+        <v>64106.05</v>
       </c>
       <c r="E80" t="n">
-        <v>-0.01</v>
+        <v>68681.05</v>
       </c>
       <c r="F80" t="n">
-        <v>0</v>
+        <v>62968.01</v>
       </c>
       <c r="G80" t="n">
-        <v>-0.01</v>
+        <v>59304.61</v>
       </c>
       <c r="H80" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="I80" t="inlineStr"/>
+        <v>332469.8</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
+          <t>13425</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="D81" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="E81" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="F81" t="n">
+        <v>-0.77</v>
+      </c>
+      <c r="G81" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="H81" t="n">
+        <v>-3.75</v>
+      </c>
+      <c r="I81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>123623963915635</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ba only</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>0</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="H82" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="I82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
           <t>90000000000000000000</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>ba only</t>
         </is>
       </c>
-      <c r="C81" t="n">
+      <c r="C83" t="n">
         <v>-0.06</v>
       </c>
-      <c r="D81" t="n">
+      <c r="D83" t="n">
         <v>-0.01</v>
       </c>
-      <c r="E81" t="n">
-        <v>0</v>
-      </c>
-      <c r="F81" t="n">
-        <v>0</v>
-      </c>
-      <c r="G81" t="n">
-        <v>0</v>
-      </c>
-      <c r="H81" t="n">
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="n">
         <v>-0.07000000000000001</v>
       </c>
-      <c r="I81" t="inlineStr"/>
+      <c r="I83" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5241,7 +5331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6953,7 +7043,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>3007</t>
+          <t>3006</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -6978,7 +7068,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>3007</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -7003,7 +7093,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -7028,7 +7118,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -7053,7 +7143,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>3333</t>
+          <t>3123</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -7062,52 +7152,48 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.71</v>
+        <v>0</v>
       </c>
       <c r="D71" t="n">
-        <v>0.41</v>
+        <v>0</v>
       </c>
       <c r="E71" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>3333</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>28500.23</v>
+        <v>0.71</v>
       </c>
       <c r="D72" t="n">
-        <v>25181.36</v>
+        <v>0.41</v>
       </c>
       <c r="E72" t="n">
-        <v>-0.01</v>
+        <v>0.48</v>
       </c>
       <c r="F72" t="n">
-        <v>53681.58</v>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
-        </is>
-      </c>
+        <v>1.6</v>
+      </c>
+      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>4011</t>
+          <t>3900</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -7127,41 +7213,41 @@
       <c r="F73" t="n">
         <v>0</v>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>4012</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>soter only</t>
+          <t>both</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>28500.23</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>25181.36</v>
       </c>
       <c r="E74" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" t="inlineStr"/>
+        <v>53681.58</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>9001</t>
+          <t>4011</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -7170,27 +7256,27 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>17730.23</v>
+        <v>0</v>
       </c>
       <c r="D75" t="n">
-        <v>14347.44</v>
+        <v>0</v>
       </c>
       <c r="E75" t="n">
-        <v>19582.45</v>
+        <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>51660.12</v>
+        <v>0</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>9998</t>
+          <t>4012</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -7215,7 +7301,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>9001</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -7224,27 +7310,27 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>373.74</v>
+        <v>17730.23</v>
       </c>
       <c r="D77" t="n">
-        <v>547.46</v>
+        <v>14347.44</v>
       </c>
       <c r="E77" t="n">
-        <v>1161.68</v>
+        <v>19582.45</v>
       </c>
       <c r="F77" t="n">
-        <v>2082.88</v>
+        <v>51660.12</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>9998</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -7253,47 +7339,101 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>77410.08</v>
+        <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>64106.05</v>
+        <v>0</v>
       </c>
       <c r="E78" t="n">
-        <v>68681.05</v>
+        <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>210197.18</v>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>soter only</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>373.74</v>
+      </c>
+      <c r="D79" t="n">
+        <v>547.46</v>
+      </c>
+      <c r="E79" t="n">
+        <v>1161.68</v>
+      </c>
+      <c r="F79" t="n">
+        <v>2082.88</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>soter only</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>77410.08</v>
+      </c>
+      <c r="D80" t="n">
+        <v>64106.05</v>
+      </c>
+      <c r="E80" t="n">
+        <v>68681.05</v>
+      </c>
+      <c r="F80" t="n">
+        <v>210197.18</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
           <t>13425</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>soter only</t>
         </is>
       </c>
-      <c r="C79" t="n">
+      <c r="C81" t="n">
         <v>858.01</v>
       </c>
-      <c r="D79" t="n">
+      <c r="D81" t="n">
         <v>774.97</v>
       </c>
-      <c r="E79" t="n">
+      <c r="E81" t="n">
         <v>858.01</v>
       </c>
-      <c r="F79" t="n">
+      <c r="F81" t="n">
         <v>2490.99</v>
       </c>
-      <c r="G79" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7334,7 +7474,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>old=133 new=145</t>
+          <t>old=133 new=148</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -7469,7 +7609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB150"/>
+  <dimension ref="A1:AB153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8982,13 +9122,13 @@
         <v>1390891.07</v>
       </c>
       <c r="Y21" t="n">
-        <v>534444.27</v>
+        <v>534443.5</v>
       </c>
       <c r="Z21" t="n">
-        <v>279380.54</v>
+        <v>279379.88</v>
       </c>
       <c r="AA21" t="n">
-        <v>22022205.51</v>
+        <v>22022204.08</v>
       </c>
       <c r="AB21" t="inlineStr">
         <is>
@@ -9148,7 +9288,7 @@
         <v>369.92</v>
       </c>
       <c r="AA24" t="n">
-        <v>91462.50999999999</v>
+        <v>91462.5</v>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
@@ -15217,12 +15357,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>3007</t>
+          <t>3006</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>sUSDS</t>
+          <t>sUSDC</t>
         </is>
       </c>
       <c r="C136" t="inlineStr"/>
@@ -15257,12 +15397,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>3007</t>
+          <t>3006</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>stUSDS</t>
+          <t>sUSDS</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
@@ -15287,17 +15427,21 @@
       <c r="V137" t="inlineStr"/>
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr"/>
-      <c r="Y137" t="inlineStr"/>
-      <c r="Z137" t="inlineStr"/>
+      <c r="Y137" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="Z137" t="n">
+        <v>0.66</v>
+      </c>
       <c r="AA137" t="n">
-        <v>0</v>
+        <v>1.43</v>
       </c>
       <c r="AB137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>3007</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -15337,12 +15481,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3007</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>sUSDS</t>
+          <t>stUSDS</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
@@ -15368,18 +15512,16 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr"/>
       <c r="Y139" t="inlineStr"/>
-      <c r="Z139" t="n">
-        <v>21.19</v>
-      </c>
+      <c r="Z139" t="inlineStr"/>
       <c r="AA139" t="n">
-        <v>21.19</v>
+        <v>0</v>
       </c>
       <c r="AB139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -15419,7 +15561,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>3333</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -15433,74 +15575,40 @@
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr"/>
-      <c r="I141" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="J141" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="K141" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="L141" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="M141" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="N141" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="O141" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="P141" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="Q141" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="R141" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="S141" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="T141" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="U141" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="V141" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="W141" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="X141" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="Y141" t="n">
-        <v>0.24</v>
-      </c>
+      <c r="I141" t="inlineStr"/>
+      <c r="J141" t="inlineStr"/>
+      <c r="K141" t="inlineStr"/>
+      <c r="L141" t="inlineStr"/>
+      <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
+      <c r="O141" t="inlineStr"/>
+      <c r="P141" t="inlineStr"/>
+      <c r="Q141" t="inlineStr"/>
+      <c r="R141" t="inlineStr"/>
+      <c r="S141" t="inlineStr"/>
+      <c r="T141" t="inlineStr"/>
+      <c r="U141" t="inlineStr"/>
+      <c r="V141" t="inlineStr"/>
+      <c r="W141" t="inlineStr"/>
+      <c r="X141" t="inlineStr"/>
+      <c r="Y141" t="inlineStr"/>
       <c r="Z141" t="n">
-        <v>0.14</v>
+        <v>21.19</v>
       </c>
       <c r="AA141" t="n">
-        <v>10.05</v>
+        <v>21.19</v>
       </c>
       <c r="AB141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>3123</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>USDS</t>
+          <t>sUSDS</t>
         </is>
       </c>
       <c r="C142" t="inlineStr"/>
@@ -15517,49 +15625,25 @@
       <c r="N142" t="inlineStr"/>
       <c r="O142" t="inlineStr"/>
       <c r="P142" t="inlineStr"/>
-      <c r="Q142" t="n">
-        <v>11499.8</v>
-      </c>
-      <c r="R142" t="n">
-        <v>33962.99</v>
-      </c>
-      <c r="S142" t="n">
-        <v>28500.23</v>
-      </c>
-      <c r="T142" t="n">
-        <v>25181.36</v>
-      </c>
-      <c r="U142" t="n">
-        <v>29061.49</v>
-      </c>
-      <c r="V142" t="n">
-        <v>23261.27</v>
-      </c>
-      <c r="W142" t="n">
-        <v>22648.4</v>
-      </c>
-      <c r="X142" t="n">
-        <v>19688.27</v>
-      </c>
-      <c r="Y142" t="n">
-        <v>4107.61</v>
-      </c>
-      <c r="Z142" t="n">
-        <v>1523.19</v>
-      </c>
+      <c r="Q142" t="inlineStr"/>
+      <c r="R142" t="inlineStr"/>
+      <c r="S142" t="inlineStr"/>
+      <c r="T142" t="inlineStr"/>
+      <c r="U142" t="inlineStr"/>
+      <c r="V142" t="inlineStr"/>
+      <c r="W142" t="inlineStr"/>
+      <c r="X142" t="inlineStr"/>
+      <c r="Y142" t="inlineStr"/>
+      <c r="Z142" t="inlineStr"/>
       <c r="AA142" t="n">
-        <v>199434.62</v>
-      </c>
-      <c r="AB142" t="inlineStr">
-        <is>
-          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>4011</t>
+          <t>3333</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -15573,48 +15657,74 @@
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr"/>
       <c r="H143" t="inlineStr"/>
-      <c r="I143" t="inlineStr"/>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
-      <c r="L143" t="inlineStr"/>
-      <c r="M143" t="inlineStr"/>
-      <c r="N143" t="inlineStr"/>
-      <c r="O143" t="inlineStr"/>
-      <c r="P143" t="inlineStr"/>
-      <c r="Q143" t="inlineStr"/>
-      <c r="R143" t="inlineStr"/>
-      <c r="S143" t="inlineStr"/>
-      <c r="T143" t="inlineStr"/>
-      <c r="U143" t="inlineStr"/>
-      <c r="V143" t="inlineStr"/>
+      <c r="I143" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="J143" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="K143" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="L143" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="M143" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="P143" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="Q143" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="R143" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="S143" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="T143" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="U143" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="V143" t="n">
+        <v>0.49</v>
+      </c>
       <c r="W143" t="n">
-        <v>76.34</v>
-      </c>
-      <c r="X143" t="inlineStr"/>
+        <v>0.48</v>
+      </c>
+      <c r="X143" t="n">
+        <v>0.39</v>
+      </c>
       <c r="Y143" t="n">
-        <v>119.5</v>
+        <v>0.24</v>
       </c>
       <c r="Z143" t="n">
-        <v>7.72</v>
+        <v>0.14</v>
       </c>
       <c r="AA143" t="n">
-        <v>203.56</v>
-      </c>
-      <c r="AB143" t="inlineStr">
-        <is>
-          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
-        </is>
-      </c>
+        <v>10.05</v>
+      </c>
+      <c r="AB143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>4012</t>
+          <t>3900</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>spUSDC</t>
+          <t>sUSDS</t>
         </is>
       </c>
       <c r="C144" t="inlineStr"/>
@@ -15649,7 +15759,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>9001</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -15658,88 +15768,62 @@
         </is>
       </c>
       <c r="C145" t="inlineStr"/>
-      <c r="D145" t="n">
-        <v>17212.5</v>
-      </c>
-      <c r="E145" t="n">
-        <v>42919.38</v>
-      </c>
-      <c r="F145" t="n">
-        <v>12845.31</v>
-      </c>
-      <c r="G145" t="n">
-        <v>67997.23</v>
-      </c>
-      <c r="H145" t="n">
-        <v>167617.09</v>
-      </c>
-      <c r="I145" t="n">
-        <v>193802.05</v>
-      </c>
-      <c r="J145" t="n">
-        <v>178859.66</v>
-      </c>
-      <c r="K145" t="n">
-        <v>115587.03</v>
-      </c>
-      <c r="L145" t="n">
-        <v>31496.94</v>
-      </c>
-      <c r="M145" t="n">
-        <v>12743.32</v>
-      </c>
-      <c r="N145" t="n">
-        <v>7874.47</v>
-      </c>
-      <c r="O145" t="n">
-        <v>10344.29</v>
-      </c>
-      <c r="P145" t="n">
-        <v>15618.57</v>
-      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr"/>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr"/>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
+      <c r="P145" t="inlineStr"/>
       <c r="Q145" t="n">
-        <v>16419.61</v>
+        <v>11499.8</v>
       </c>
       <c r="R145" t="n">
-        <v>24700.59</v>
+        <v>33962.99</v>
       </c>
       <c r="S145" t="n">
-        <v>17730.23</v>
+        <v>28500.23</v>
       </c>
       <c r="T145" t="n">
-        <v>14347.44</v>
+        <v>25181.36</v>
       </c>
       <c r="U145" t="n">
-        <v>19582.45</v>
+        <v>29061.49</v>
       </c>
       <c r="V145" t="n">
-        <v>15967.76</v>
+        <v>23261.27</v>
       </c>
       <c r="W145" t="n">
-        <v>9527.389999999999</v>
+        <v>22648.4</v>
       </c>
       <c r="X145" t="n">
-        <v>5835.14</v>
+        <v>19688.27</v>
       </c>
       <c r="Y145" t="n">
-        <v>2750.87</v>
+        <v>4107.61</v>
       </c>
       <c r="Z145" t="n">
-        <v>1993.6</v>
+        <v>1523.19</v>
       </c>
       <c r="AA145" t="n">
-        <v>1003772.92</v>
+        <v>199434.62</v>
       </c>
       <c r="AB145" t="inlineStr">
         <is>
-          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>9998</t>
+          <t>4011</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -15757,13 +15841,9 @@
       <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr"/>
-      <c r="M146" t="n">
-        <v>0.01</v>
-      </c>
+      <c r="M146" t="inlineStr"/>
       <c r="N146" t="inlineStr"/>
-      <c r="O146" t="n">
-        <v>3.79</v>
-      </c>
+      <c r="O146" t="inlineStr"/>
       <c r="P146" t="inlineStr"/>
       <c r="Q146" t="inlineStr"/>
       <c r="R146" t="inlineStr"/>
@@ -15771,196 +15851,168 @@
       <c r="T146" t="inlineStr"/>
       <c r="U146" t="inlineStr"/>
       <c r="V146" t="inlineStr"/>
-      <c r="W146" t="inlineStr"/>
+      <c r="W146" t="n">
+        <v>76.34</v>
+      </c>
       <c r="X146" t="inlineStr"/>
-      <c r="Y146" t="inlineStr"/>
-      <c r="Z146" t="inlineStr"/>
+      <c r="Y146" t="n">
+        <v>119.5</v>
+      </c>
+      <c r="Z146" t="n">
+        <v>7.72</v>
+      </c>
       <c r="AA146" t="n">
-        <v>3.81</v>
-      </c>
-      <c r="AB146" t="inlineStr"/>
+        <v>203.56</v>
+      </c>
+      <c r="AB146" t="inlineStr">
+        <is>
+          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>4012</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>sUSDS</t>
+          <t>spUSDC</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr"/>
       <c r="E147" t="inlineStr"/>
-      <c r="F147" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="G147" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="H147" t="n">
-        <v>60.32</v>
-      </c>
-      <c r="I147" t="n">
-        <v>843.76</v>
-      </c>
-      <c r="J147" t="n">
-        <v>225.41</v>
-      </c>
-      <c r="K147" t="n">
-        <v>108.13</v>
-      </c>
-      <c r="L147" t="n">
-        <v>98.39</v>
-      </c>
-      <c r="M147" t="n">
-        <v>111.81</v>
-      </c>
-      <c r="N147" t="n">
-        <v>139.45</v>
-      </c>
-      <c r="O147" t="n">
-        <v>100.56</v>
-      </c>
-      <c r="P147" t="n">
-        <v>53.73</v>
-      </c>
-      <c r="Q147" t="n">
-        <v>38.36</v>
-      </c>
-      <c r="R147" t="n">
-        <v>38.81</v>
-      </c>
-      <c r="S147" t="n">
-        <v>373.74</v>
-      </c>
-      <c r="T147" t="n">
-        <v>547.46</v>
-      </c>
-      <c r="U147" t="n">
-        <v>1161.68</v>
-      </c>
-      <c r="V147" t="n">
-        <v>1570.26</v>
-      </c>
-      <c r="W147" t="n">
-        <v>1039.27</v>
-      </c>
-      <c r="X147" t="n">
-        <v>734.97</v>
-      </c>
-      <c r="Y147" t="n">
-        <v>419.53</v>
-      </c>
-      <c r="Z147" t="n">
-        <v>179.36</v>
-      </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr"/>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr"/>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
+      <c r="P147" t="inlineStr"/>
+      <c r="Q147" t="inlineStr"/>
+      <c r="R147" t="inlineStr"/>
+      <c r="S147" t="inlineStr"/>
+      <c r="T147" t="inlineStr"/>
+      <c r="U147" t="inlineStr"/>
+      <c r="V147" t="inlineStr"/>
+      <c r="W147" t="inlineStr"/>
+      <c r="X147" t="inlineStr"/>
+      <c r="Y147" t="inlineStr"/>
+      <c r="Z147" t="inlineStr"/>
       <c r="AA147" t="n">
-        <v>7846.25</v>
-      </c>
-      <c r="AB147" t="inlineStr">
-        <is>
-          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AB147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>9001</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>sUSDS</t>
+          <t>USDS</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
-      <c r="D148" t="inlineStr"/>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
-      <c r="H148" t="inlineStr"/>
+      <c r="D148" t="n">
+        <v>17212.5</v>
+      </c>
+      <c r="E148" t="n">
+        <v>42919.38</v>
+      </c>
+      <c r="F148" t="n">
+        <v>12845.31</v>
+      </c>
+      <c r="G148" t="n">
+        <v>67997.23</v>
+      </c>
+      <c r="H148" t="n">
+        <v>167617.09</v>
+      </c>
       <c r="I148" t="n">
-        <v>2043.15</v>
+        <v>193802.05</v>
       </c>
       <c r="J148" t="n">
-        <v>6732.26</v>
+        <v>178859.66</v>
       </c>
       <c r="K148" t="n">
-        <v>11662.59</v>
+        <v>115587.03</v>
       </c>
       <c r="L148" t="n">
-        <v>43973.92</v>
+        <v>31496.94</v>
       </c>
       <c r="M148" t="n">
-        <v>37718.86</v>
+        <v>12743.32</v>
       </c>
       <c r="N148" t="n">
-        <v>48771.92</v>
+        <v>7874.47</v>
       </c>
       <c r="O148" t="n">
-        <v>66723.57000000001</v>
+        <v>10344.29</v>
       </c>
       <c r="P148" t="n">
-        <v>70944.55</v>
+        <v>15618.57</v>
       </c>
       <c r="Q148" t="n">
-        <v>70839.37</v>
+        <v>16419.61</v>
       </c>
       <c r="R148" t="n">
-        <v>92454.63</v>
+        <v>24700.59</v>
       </c>
       <c r="S148" t="n">
-        <v>77410.08</v>
+        <v>17730.23</v>
       </c>
       <c r="T148" t="n">
-        <v>64106.05</v>
+        <v>14347.44</v>
       </c>
       <c r="U148" t="n">
-        <v>68681.05</v>
+        <v>19582.45</v>
       </c>
       <c r="V148" t="n">
-        <v>62968.01</v>
+        <v>15967.76</v>
       </c>
       <c r="W148" t="n">
-        <v>59304.61</v>
+        <v>9527.389999999999</v>
       </c>
       <c r="X148" t="n">
-        <v>56940.63</v>
+        <v>5835.14</v>
       </c>
       <c r="Y148" t="n">
-        <v>36971.31</v>
+        <v>2750.87</v>
       </c>
       <c r="Z148" t="n">
-        <v>35115.46</v>
+        <v>1993.6</v>
       </c>
       <c r="AA148" t="n">
-        <v>913362.02</v>
+        <v>1003772.92</v>
       </c>
       <c r="AB148" t="inlineStr">
         <is>
-          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
+          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>13425</t>
+          <t>9998</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>USDS-SKY</t>
+          <t>sUSDS</t>
         </is>
       </c>
       <c r="C149" t="inlineStr"/>
-      <c r="D149" t="n">
-        <v>0.03</v>
-      </c>
+      <c r="D149" t="inlineStr"/>
       <c r="E149" t="inlineStr"/>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr"/>
@@ -15969,100 +16021,312 @@
       <c r="J149" t="inlineStr"/>
       <c r="K149" t="inlineStr"/>
       <c r="L149" t="inlineStr"/>
-      <c r="M149" t="inlineStr"/>
+      <c r="M149" t="n">
+        <v>0.01</v>
+      </c>
       <c r="N149" t="inlineStr"/>
-      <c r="O149" t="inlineStr"/>
+      <c r="O149" t="n">
+        <v>3.79</v>
+      </c>
       <c r="P149" t="inlineStr"/>
-      <c r="Q149" t="n">
-        <v>370.4</v>
-      </c>
-      <c r="R149" t="n">
-        <v>1029.1</v>
-      </c>
-      <c r="S149" t="n">
-        <v>858.01</v>
-      </c>
-      <c r="T149" t="n">
-        <v>774.97</v>
-      </c>
-      <c r="U149" t="n">
-        <v>858.01</v>
-      </c>
-      <c r="V149" t="n">
-        <v>641.16</v>
-      </c>
-      <c r="W149" t="n">
-        <v>9.67</v>
-      </c>
-      <c r="X149" t="n">
-        <v>9.359999999999999</v>
-      </c>
-      <c r="Y149" t="n">
-        <v>5.37</v>
-      </c>
-      <c r="Z149" t="n">
-        <v>3.87</v>
-      </c>
+      <c r="Q149" t="inlineStr"/>
+      <c r="R149" t="inlineStr"/>
+      <c r="S149" t="inlineStr"/>
+      <c r="T149" t="inlineStr"/>
+      <c r="U149" t="inlineStr"/>
+      <c r="V149" t="inlineStr"/>
+      <c r="W149" t="inlineStr"/>
+      <c r="X149" t="inlineStr"/>
+      <c r="Y149" t="inlineStr"/>
+      <c r="Z149" t="inlineStr"/>
       <c r="AA149" t="n">
-        <v>4559.96</v>
+        <v>3.81</v>
       </c>
       <c r="AB149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>sUSDS</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G150" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="H150" t="n">
+        <v>60.32</v>
+      </c>
+      <c r="I150" t="n">
+        <v>843.76</v>
+      </c>
+      <c r="J150" t="n">
+        <v>225.41</v>
+      </c>
+      <c r="K150" t="n">
+        <v>108.13</v>
+      </c>
+      <c r="L150" t="n">
+        <v>98.39</v>
+      </c>
+      <c r="M150" t="n">
+        <v>111.81</v>
+      </c>
+      <c r="N150" t="n">
+        <v>139.45</v>
+      </c>
+      <c r="O150" t="n">
+        <v>100.56</v>
+      </c>
+      <c r="P150" t="n">
+        <v>53.73</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>38.36</v>
+      </c>
+      <c r="R150" t="n">
+        <v>38.81</v>
+      </c>
+      <c r="S150" t="n">
+        <v>373.74</v>
+      </c>
+      <c r="T150" t="n">
+        <v>547.46</v>
+      </c>
+      <c r="U150" t="n">
+        <v>1161.68</v>
+      </c>
+      <c r="V150" t="n">
+        <v>1570.26</v>
+      </c>
+      <c r="W150" t="n">
+        <v>1039.27</v>
+      </c>
+      <c r="X150" t="n">
+        <v>734.97</v>
+      </c>
+      <c r="Y150" t="n">
+        <v>419.53</v>
+      </c>
+      <c r="Z150" t="n">
+        <v>179.36</v>
+      </c>
+      <c r="AA150" t="n">
+        <v>7846.25</v>
+      </c>
+      <c r="AB150" t="inlineStr">
+        <is>
+          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>sUSDS</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="n">
+        <v>2043.15</v>
+      </c>
+      <c r="J151" t="n">
+        <v>6732.26</v>
+      </c>
+      <c r="K151" t="n">
+        <v>11662.59</v>
+      </c>
+      <c r="L151" t="n">
+        <v>43973.92</v>
+      </c>
+      <c r="M151" t="n">
+        <v>37718.86</v>
+      </c>
+      <c r="N151" t="n">
+        <v>48771.92</v>
+      </c>
+      <c r="O151" t="n">
+        <v>66723.57000000001</v>
+      </c>
+      <c r="P151" t="n">
+        <v>70944.55</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>70839.37</v>
+      </c>
+      <c r="R151" t="n">
+        <v>92454.63</v>
+      </c>
+      <c r="S151" t="n">
+        <v>77410.08</v>
+      </c>
+      <c r="T151" t="n">
+        <v>64106.05</v>
+      </c>
+      <c r="U151" t="n">
+        <v>68681.05</v>
+      </c>
+      <c r="V151" t="n">
+        <v>62968.01</v>
+      </c>
+      <c r="W151" t="n">
+        <v>59304.61</v>
+      </c>
+      <c r="X151" t="n">
+        <v>56940.63</v>
+      </c>
+      <c r="Y151" t="n">
+        <v>36971.31</v>
+      </c>
+      <c r="Z151" t="n">
+        <v>35115.46</v>
+      </c>
+      <c r="AA151" t="n">
+        <v>913362.02</v>
+      </c>
+      <c r="AB151" t="inlineStr">
+        <is>
+          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
           <t>13425</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>USDS-SKY</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr"/>
+      <c r="M152" t="inlineStr"/>
+      <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr"/>
+      <c r="P152" t="inlineStr"/>
+      <c r="Q152" t="n">
+        <v>370.4</v>
+      </c>
+      <c r="R152" t="n">
+        <v>1029.1</v>
+      </c>
+      <c r="S152" t="n">
+        <v>858.01</v>
+      </c>
+      <c r="T152" t="n">
+        <v>774.97</v>
+      </c>
+      <c r="U152" t="n">
+        <v>858.01</v>
+      </c>
+      <c r="V152" t="n">
+        <v>641.16</v>
+      </c>
+      <c r="W152" t="n">
+        <v>9.67</v>
+      </c>
+      <c r="X152" t="n">
+        <v>9.359999999999999</v>
+      </c>
+      <c r="Y152" t="n">
+        <v>5.37</v>
+      </c>
+      <c r="Z152" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="AA152" t="n">
+        <v>4559.96</v>
+      </c>
+      <c r="AB152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>13425</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
         <is>
           <t>sUSDS</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr"/>
-      <c r="D150" t="n">
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="n">
         <v>0.14</v>
       </c>
-      <c r="E150" t="n">
+      <c r="E153" t="n">
         <v>0.18</v>
       </c>
-      <c r="F150" t="n">
+      <c r="F153" t="n">
         <v>0.18</v>
       </c>
-      <c r="G150" t="n">
+      <c r="G153" t="n">
         <v>0.19</v>
       </c>
-      <c r="H150" t="n">
+      <c r="H153" t="n">
         <v>0.17</v>
       </c>
-      <c r="I150" t="n">
+      <c r="I153" t="n">
         <v>0.19</v>
       </c>
-      <c r="J150" t="n">
+      <c r="J153" t="n">
         <v>0.18</v>
       </c>
-      <c r="K150" t="n">
+      <c r="K153" t="n">
         <v>0.1</v>
       </c>
-      <c r="L150" t="inlineStr"/>
-      <c r="M150" t="inlineStr"/>
-      <c r="N150" t="inlineStr"/>
-      <c r="O150" t="inlineStr"/>
-      <c r="P150" t="inlineStr"/>
-      <c r="Q150" t="inlineStr"/>
-      <c r="R150" t="inlineStr"/>
-      <c r="S150" t="inlineStr"/>
-      <c r="T150" t="inlineStr"/>
-      <c r="U150" t="inlineStr"/>
-      <c r="V150" t="inlineStr"/>
-      <c r="W150" t="inlineStr"/>
-      <c r="X150" t="inlineStr"/>
-      <c r="Y150" t="inlineStr"/>
-      <c r="Z150" t="inlineStr"/>
-      <c r="AA150" t="n">
+      <c r="L153" t="inlineStr"/>
+      <c r="M153" t="inlineStr"/>
+      <c r="N153" t="inlineStr"/>
+      <c r="O153" t="inlineStr"/>
+      <c r="P153" t="inlineStr"/>
+      <c r="Q153" t="inlineStr"/>
+      <c r="R153" t="inlineStr"/>
+      <c r="S153" t="inlineStr"/>
+      <c r="T153" t="inlineStr"/>
+      <c r="U153" t="inlineStr"/>
+      <c r="V153" t="inlineStr"/>
+      <c r="W153" t="inlineStr"/>
+      <c r="X153" t="inlineStr"/>
+      <c r="Y153" t="inlineStr"/>
+      <c r="Z153" t="inlineStr"/>
+      <c r="AA153" t="n">
         <v>1.33</v>
       </c>
-      <c r="AB150" t="inlineStr"/>
+      <c r="AB153" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16075,7 +16339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N62"/>
+  <dimension ref="A1:N63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18217,7 +18481,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3006</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -18236,12 +18500,14 @@
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
+      <c r="J49" t="n">
+        <v>0.77</v>
+      </c>
       <c r="K49" t="n">
-        <v>21.19</v>
+        <v>0.66</v>
       </c>
       <c r="L49" t="n">
-        <v>21.19</v>
+        <v>1.43</v>
       </c>
       <c r="M49" t="n">
         <v>0</v>
@@ -18251,7 +18517,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>3333</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -18264,42 +18530,28 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>0.71</v>
-      </c>
-      <c r="E50" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="F50" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="G50" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="H50" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="I50" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="J50" t="n">
-        <v>0.24</v>
-      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
       <c r="K50" t="n">
-        <v>0.14</v>
+        <v>21.19</v>
       </c>
       <c r="L50" t="n">
-        <v>3.35</v>
+        <v>21.19</v>
       </c>
       <c r="M50" t="n">
-        <v>6.7</v>
+        <v>0</v>
       </c>
       <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>3333</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -18313,45 +18565,41 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>28500.23</v>
+        <v>0.71</v>
       </c>
       <c r="E51" t="n">
-        <v>25181.36</v>
+        <v>0.41</v>
       </c>
       <c r="F51" t="n">
-        <v>29061.49</v>
+        <v>0.48</v>
       </c>
       <c r="G51" t="n">
-        <v>23261.27</v>
+        <v>0.49</v>
       </c>
       <c r="H51" t="n">
-        <v>22648.4</v>
+        <v>0.48</v>
       </c>
       <c r="I51" t="n">
-        <v>19688.27</v>
+        <v>0.39</v>
       </c>
       <c r="J51" t="n">
-        <v>4107.61</v>
+        <v>0.24</v>
       </c>
       <c r="K51" t="n">
-        <v>1523.19</v>
+        <v>0.14</v>
       </c>
       <c r="L51" t="n">
-        <v>153971.83</v>
+        <v>3.35</v>
       </c>
       <c r="M51" t="n">
-        <v>45462.79</v>
-      </c>
-      <c r="N51" t="inlineStr">
-        <is>
-          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
-        </is>
-      </c>
+        <v>6.7</v>
+      </c>
+      <c r="N51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>4011</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -18364,36 +18612,46 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
+      <c r="D52" t="n">
+        <v>28500.23</v>
+      </c>
+      <c r="E52" t="n">
+        <v>25181.36</v>
+      </c>
+      <c r="F52" t="n">
+        <v>29061.49</v>
+      </c>
+      <c r="G52" t="n">
+        <v>23261.27</v>
+      </c>
       <c r="H52" t="n">
-        <v>76.34</v>
-      </c>
-      <c r="I52" t="inlineStr"/>
+        <v>22648.4</v>
+      </c>
+      <c r="I52" t="n">
+        <v>19688.27</v>
+      </c>
       <c r="J52" t="n">
-        <v>119.5</v>
+        <v>4107.61</v>
       </c>
       <c r="K52" t="n">
-        <v>7.72</v>
+        <v>1523.19</v>
       </c>
       <c r="L52" t="n">
-        <v>203.56</v>
+        <v>153971.83</v>
       </c>
       <c r="M52" t="n">
-        <v>0</v>
+        <v>45462.79</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
-          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
+          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>9001</t>
+          <t>4011</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -18406,46 +18664,36 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>17730.23</v>
-      </c>
-      <c r="E53" t="n">
-        <v>14347.44</v>
-      </c>
-      <c r="F53" t="n">
-        <v>19582.45</v>
-      </c>
-      <c r="G53" t="n">
-        <v>15967.76</v>
-      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
       <c r="H53" t="n">
-        <v>9527.389999999999</v>
-      </c>
-      <c r="I53" t="n">
-        <v>5835.14</v>
-      </c>
+        <v>76.34</v>
+      </c>
+      <c r="I53" t="inlineStr"/>
       <c r="J53" t="n">
-        <v>2750.87</v>
+        <v>119.5</v>
       </c>
       <c r="K53" t="n">
-        <v>1993.6</v>
+        <v>7.72</v>
       </c>
       <c r="L53" t="n">
-        <v>87734.86</v>
+        <v>203.56</v>
       </c>
       <c r="M53" t="n">
-        <v>916038.0600000001</v>
+        <v>0</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>9998</t>
+          <t>9001</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -18458,148 +18706,150 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
+      <c r="D54" t="n">
+        <v>17730.23</v>
+      </c>
+      <c r="E54" t="n">
+        <v>14347.44</v>
+      </c>
+      <c r="F54" t="n">
+        <v>19582.45</v>
+      </c>
+      <c r="G54" t="n">
+        <v>15967.76</v>
+      </c>
+      <c r="H54" t="n">
+        <v>9527.389999999999</v>
+      </c>
+      <c r="I54" t="n">
+        <v>5835.14</v>
+      </c>
+      <c r="J54" t="n">
+        <v>2750.87</v>
+      </c>
+      <c r="K54" t="n">
+        <v>1993.6</v>
+      </c>
       <c r="L54" t="n">
-        <v>0.01</v>
+        <v>87734.86</v>
       </c>
       <c r="M54" t="n">
-        <v>3.81</v>
-      </c>
-      <c r="N54" t="inlineStr"/>
+        <v>916038.0600000001</v>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>9998</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="inlineStr"/>
+      <c r="L55" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="M55" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="N55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>13425</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>2026-01</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D55" t="n">
+      <c r="D56" t="n">
         <v>858.01</v>
       </c>
-      <c r="E55" t="n">
+      <c r="E56" t="n">
         <v>774.97</v>
       </c>
-      <c r="F55" t="n">
+      <c r="F56" t="n">
         <v>858.01</v>
       </c>
-      <c r="G55" t="n">
+      <c r="G56" t="n">
         <v>641.16</v>
       </c>
-      <c r="H55" t="n">
+      <c r="H56" t="n">
         <v>9.67</v>
       </c>
-      <c r="I55" t="n">
+      <c r="I56" t="n">
         <v>9.359999999999999</v>
       </c>
-      <c r="J55" t="n">
+      <c r="J56" t="n">
         <v>5.37</v>
       </c>
-      <c r="K55" t="n">
+      <c r="K56" t="n">
         <v>3.87</v>
       </c>
-      <c r="L55" t="n">
+      <c r="L56" t="n">
         <v>3160.42</v>
       </c>
-      <c r="M55" t="n">
+      <c r="M56" t="n">
         <v>1400.86</v>
       </c>
-      <c r="N55" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>SYNTHETIC &amp; UNPAID (tracked, no beneficiary — notional dr_usd; never pay, never in the payment spreadsheet)</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
-      <c r="L57" t="inlineStr"/>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>all-time total</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>-999999</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D58" t="n">
-        <v>14618.04</v>
-      </c>
-      <c r="E58" t="n">
-        <v>9853.139999999999</v>
-      </c>
-      <c r="F58" t="n">
-        <v>14833.94</v>
-      </c>
-      <c r="G58" t="n">
-        <v>8671.389999999999</v>
-      </c>
-      <c r="H58" t="n">
-        <v>7872.29</v>
-      </c>
-      <c r="I58" t="n">
-        <v>7369.06</v>
-      </c>
-      <c r="J58" t="n">
-        <v>5533.84</v>
-      </c>
-      <c r="K58" t="n">
-        <v>4420.98</v>
-      </c>
+          <t>SYNTHETIC &amp; UNPAID (tracked, no beneficiary — notional dr_usd; never pay, never in the payment spreadsheet)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr"/>
+      <c r="C58" t="inlineStr"/>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
-      <c r="M58" t="n">
-        <v>1092599.94</v>
-      </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>Synthetic code: Untagged USDS-CLE, USDS-SKY, USDS-SPK, stUSDS.</t>
-        </is>
-      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>all-time total</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>-999999</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -18613,43 +18863,43 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1199152.68</v>
+        <v>14618.04</v>
       </c>
       <c r="E59" t="n">
-        <v>1325197.22</v>
+        <v>9853.139999999999</v>
       </c>
       <c r="F59" t="n">
-        <v>1488079.24</v>
+        <v>14833.94</v>
       </c>
       <c r="G59" t="n">
-        <v>1497865.34</v>
+        <v>8671.389999999999</v>
       </c>
       <c r="H59" t="n">
-        <v>1740557.11</v>
+        <v>7872.29</v>
       </c>
       <c r="I59" t="n">
-        <v>1390891.07</v>
+        <v>7369.06</v>
       </c>
       <c r="J59" t="n">
-        <v>534444.27</v>
+        <v>5533.84</v>
       </c>
       <c r="K59" t="n">
-        <v>279380.54</v>
+        <v>4420.98</v>
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="n">
-        <v>22022205.51</v>
+        <v>1092599.94</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>Synthetic code: Untagged sUSDS.</t>
+          <t>Synthetic code: Untagged USDS-CLE, USDS-SKY, USDS-SPK, stUSDS.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -18663,43 +18913,43 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>7581.55</v>
+        <v>1199152.68</v>
       </c>
       <c r="E60" t="n">
-        <v>6588.11</v>
+        <v>1325197.22</v>
       </c>
       <c r="F60" t="n">
-        <v>5410.52</v>
+        <v>1488079.24</v>
       </c>
       <c r="G60" t="n">
-        <v>3613.36</v>
+        <v>1497865.34</v>
       </c>
       <c r="H60" t="n">
-        <v>1824.59</v>
+        <v>1740557.11</v>
       </c>
       <c r="I60" t="n">
-        <v>5924.87</v>
+        <v>1390891.07</v>
       </c>
       <c r="J60" t="n">
-        <v>2653.18</v>
+        <v>534443.5</v>
       </c>
       <c r="K60" t="n">
-        <v>369.92</v>
+        <v>279379.88</v>
       </c>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="n">
-        <v>91462.50999999999</v>
+        <v>22022204.08</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>Synthetic code: untagged sUSDC</t>
+          <t>Synthetic code: Untagged sUSDS.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>127</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -18713,43 +18963,43 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>373.74</v>
+        <v>7581.55</v>
       </c>
       <c r="E61" t="n">
-        <v>547.46</v>
+        <v>6588.11</v>
       </c>
       <c r="F61" t="n">
-        <v>1161.68</v>
+        <v>5410.52</v>
       </c>
       <c r="G61" t="n">
-        <v>1570.26</v>
+        <v>3613.36</v>
       </c>
       <c r="H61" t="n">
-        <v>1039.27</v>
+        <v>1824.59</v>
       </c>
       <c r="I61" t="n">
-        <v>734.97</v>
+        <v>5924.87</v>
       </c>
       <c r="J61" t="n">
-        <v>419.53</v>
+        <v>2653.18</v>
       </c>
       <c r="K61" t="n">
-        <v>179.36</v>
+        <v>369.92</v>
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="n">
-        <v>7846.25</v>
+        <v>91462.5</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
-          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+          <t>Synthetic code: untagged sUSDC</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -18763,34 +19013,84 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>77410.08</v>
+        <v>373.74</v>
       </c>
       <c r="E62" t="n">
-        <v>64106.05</v>
+        <v>547.46</v>
       </c>
       <c r="F62" t="n">
-        <v>68681.05</v>
+        <v>1161.68</v>
       </c>
       <c r="G62" t="n">
-        <v>62968.01</v>
+        <v>1570.26</v>
       </c>
       <c r="H62" t="n">
-        <v>59304.61</v>
+        <v>1039.27</v>
       </c>
       <c r="I62" t="n">
-        <v>56940.63</v>
+        <v>734.97</v>
       </c>
       <c r="J62" t="n">
-        <v>36971.31</v>
+        <v>419.53</v>
       </c>
       <c r="K62" t="n">
-        <v>35115.46</v>
+        <v>179.36</v>
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="n">
+        <v>7846.25</v>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>77410.08</v>
+      </c>
+      <c r="E63" t="n">
+        <v>64106.05</v>
+      </c>
+      <c r="F63" t="n">
+        <v>68681.05</v>
+      </c>
+      <c r="G63" t="n">
+        <v>62968.01</v>
+      </c>
+      <c r="H63" t="n">
+        <v>59304.61</v>
+      </c>
+      <c r="I63" t="n">
+        <v>56940.63</v>
+      </c>
+      <c r="J63" t="n">
+        <v>36971.31</v>
+      </c>
+      <c r="K63" t="n">
+        <v>35115.46</v>
+      </c>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="n">
         <v>913362.02</v>
       </c>
-      <c r="N62" t="inlineStr">
+      <c r="N63" t="inlineStr">
         <is>
           <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
         </is>
@@ -22583,7 +22883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24929,12 +25229,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>3007</t>
+          <t>3006</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -24963,7 +25263,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>3007</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -24997,12 +25297,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>soter only</t>
+          <t>both</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -25031,7 +25331,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -25065,12 +25365,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>3333</t>
+          <t>3123</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -25083,13 +25383,13 @@
         <v>0</v>
       </c>
       <c r="F72" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G72" t="n">
         <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
         <v>0</v>
@@ -25099,50 +25399,46 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>3333</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>soter only</t>
+          <t>both</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>28500.23</v>
+        <v>0</v>
       </c>
       <c r="D73" t="n">
-        <v>25181.36</v>
+        <v>0</v>
       </c>
       <c r="E73" t="n">
-        <v>29061.49</v>
+        <v>0</v>
       </c>
       <c r="F73" t="n">
-        <v>23261.27</v>
+        <v>-0</v>
       </c>
       <c r="G73" t="n">
-        <v>22648.4</v>
+        <v>0</v>
       </c>
       <c r="H73" t="n">
-        <v>19688.27</v>
+        <v>-0</v>
       </c>
       <c r="I73" t="n">
-        <v>148341.02</v>
-      </c>
-      <c r="J73" t="inlineStr">
-        <is>
-          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>4011</t>
+          <t>3900</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -25158,96 +25454,96 @@
         <v>0</v>
       </c>
       <c r="G74" t="n">
-        <v>76.33</v>
+        <v>0</v>
       </c>
       <c r="H74" t="n">
         <v>0</v>
       </c>
       <c r="I74" t="n">
-        <v>76.33</v>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>4012</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>0</v>
+        <v>28500.23</v>
       </c>
       <c r="D75" t="n">
-        <v>0</v>
+        <v>25181.36</v>
       </c>
       <c r="E75" t="n">
-        <v>0</v>
+        <v>29061.49</v>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
+        <v>23261.27</v>
       </c>
       <c r="G75" t="n">
-        <v>0</v>
+        <v>22648.4</v>
       </c>
       <c r="H75" t="n">
-        <v>0</v>
+        <v>19688.27</v>
       </c>
       <c r="I75" t="n">
-        <v>0</v>
-      </c>
-      <c r="J75" t="inlineStr"/>
+        <v>148341.02</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>9001</t>
+          <t>4011</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>soter only</t>
+          <t>both</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>17730.23</v>
+        <v>0</v>
       </c>
       <c r="D76" t="n">
-        <v>14347.44</v>
+        <v>0</v>
       </c>
       <c r="E76" t="n">
-        <v>19582.45</v>
+        <v>0</v>
       </c>
       <c r="F76" t="n">
-        <v>15967.76</v>
+        <v>0</v>
       </c>
       <c r="G76" t="n">
-        <v>9527.389999999999</v>
+        <v>76.33</v>
       </c>
       <c r="H76" t="n">
-        <v>5835.14</v>
+        <v>0</v>
       </c>
       <c r="I76" t="n">
-        <v>82990.41</v>
+        <v>76.33</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>9998</t>
+          <t>4012</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -25281,7 +25577,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>9001</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -25290,171 +25586,243 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>373.74</v>
+        <v>17730.23</v>
       </c>
       <c r="D78" t="n">
-        <v>547.46</v>
+        <v>14347.44</v>
       </c>
       <c r="E78" t="n">
-        <v>1161.68</v>
+        <v>19582.45</v>
       </c>
       <c r="F78" t="n">
-        <v>1570.26</v>
+        <v>15967.76</v>
       </c>
       <c r="G78" t="n">
-        <v>1039.27</v>
+        <v>9527.389999999999</v>
       </c>
       <c r="H78" t="n">
-        <v>734.97</v>
+        <v>5835.14</v>
       </c>
       <c r="I78" t="n">
-        <v>5427.38</v>
+        <v>82990.41</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>9998</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>soter only</t>
+          <t>both</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>77410.08</v>
+        <v>0</v>
       </c>
       <c r="D79" t="n">
-        <v>64106.05</v>
+        <v>0</v>
       </c>
       <c r="E79" t="n">
-        <v>68681.05</v>
+        <v>0</v>
       </c>
       <c r="F79" t="n">
-        <v>62968.01</v>
+        <v>0</v>
       </c>
       <c r="G79" t="n">
-        <v>59304.61</v>
+        <v>0</v>
       </c>
       <c r="H79" t="n">
-        <v>56940.63</v>
+        <v>0</v>
       </c>
       <c r="I79" t="n">
-        <v>389410.43</v>
-      </c>
-      <c r="J79" t="inlineStr">
-        <is>
-          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>13425</t>
+          <t>10000</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>both</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>-0</v>
+        <v>373.74</v>
       </c>
       <c r="D80" t="n">
-        <v>0</v>
+        <v>547.46</v>
       </c>
       <c r="E80" t="n">
-        <v>0</v>
+        <v>1161.68</v>
       </c>
       <c r="F80" t="n">
-        <v>0</v>
+        <v>1570.26</v>
       </c>
       <c r="G80" t="n">
-        <v>-0</v>
+        <v>1039.27</v>
       </c>
       <c r="H80" t="n">
-        <v>-0</v>
+        <v>734.97</v>
       </c>
       <c r="I80" t="n">
-        <v>0</v>
-      </c>
-      <c r="J80" t="inlineStr"/>
+        <v>5427.38</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>123623963915635</t>
+          <t>10001</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>spark only</t>
+          <t>soter only</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>0</v>
+        <v>77410.08</v>
       </c>
       <c r="D81" t="n">
-        <v>0</v>
+        <v>64106.05</v>
       </c>
       <c r="E81" t="n">
-        <v>-0.01</v>
+        <v>68681.05</v>
       </c>
       <c r="F81" t="n">
-        <v>0</v>
+        <v>62968.01</v>
       </c>
       <c r="G81" t="n">
-        <v>-0.01</v>
+        <v>59304.61</v>
       </c>
       <c r="H81" t="n">
-        <v>0</v>
+        <v>56940.63</v>
       </c>
       <c r="I81" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="J81" t="inlineStr"/>
+        <v>389410.43</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>13425</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H82" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>123623963915635</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>spark only</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" t="n">
+        <v>0</v>
+      </c>
+      <c r="E83" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="J83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t>90000000000000000000</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>spark only</t>
         </is>
       </c>
-      <c r="C82" t="n">
+      <c r="C84" t="n">
         <v>-0.06</v>
       </c>
-      <c r="D82" t="n">
+      <c r="D84" t="n">
         <v>-0.01</v>
       </c>
-      <c r="E82" t="n">
-        <v>0</v>
-      </c>
-      <c r="F82" t="n">
-        <v>0</v>
-      </c>
-      <c r="G82" t="n">
-        <v>0</v>
-      </c>
-      <c r="H82" t="n">
-        <v>0</v>
-      </c>
-      <c r="I82" t="n">
+      <c r="E84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" t="n">
         <v>-0.07000000000000001</v>
       </c>
-      <c r="J82" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25467,7 +25835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G79"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27179,7 +27547,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>3007</t>
+          <t>3006</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -27204,7 +27572,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>3008</t>
+          <t>3007</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -27229,7 +27597,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>3009</t>
+          <t>3008</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -27254,7 +27622,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>3123</t>
+          <t>3009</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -27279,7 +27647,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>3333</t>
+          <t>3123</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -27288,23 +27656,23 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.71</v>
+        <v>0</v>
       </c>
       <c r="D71" t="n">
-        <v>0.41</v>
+        <v>0</v>
       </c>
       <c r="E71" t="n">
-        <v>0.48</v>
+        <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>1.6</v>
+        <v>0</v>
       </c>
       <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>4001</t>
+          <t>3333</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -27313,27 +27681,23 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>28500.23</v>
+        <v>0.71</v>
       </c>
       <c r="D72" t="n">
-        <v>25181.36</v>
+        <v>0.41</v>
       </c>
       <c r="E72" t="n">
-        <v>29061.49</v>
+        <v>0.48</v>
       </c>
       <c r="F72" t="n">
-        <v>82743.08</v>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
-        </is>
-      </c>
+        <v>1.6</v>
+      </c>
+      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>4011</t>
+          <t>3900</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -27353,16 +27717,12 @@
       <c r="F73" t="n">
         <v>0</v>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>4012</t>
+          <t>4001</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -27371,23 +27731,27 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>0</v>
+        <v>28500.23</v>
       </c>
       <c r="D74" t="n">
-        <v>0</v>
+        <v>25181.36</v>
       </c>
       <c r="E74" t="n">
-        <v>0</v>
+        <v>29061.49</v>
       </c>
       <c r="F74" t="n">
-        <v>0</v>
-      </c>
-      <c r="G74" t="inlineStr"/>
+        <v>82743.08</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Synthetic code: USDS in Solana OFT Bridge; entire contract balance. Intraday TWA (clean methodology; Dune query used EOD snapshots).</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>9001</t>
+          <t>4011</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -27396,27 +27760,27 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>17730.23</v>
+        <v>0</v>
       </c>
       <c r="D75" t="n">
-        <v>14347.44</v>
+        <v>0</v>
       </c>
       <c r="E75" t="n">
-        <v>19582.45</v>
+        <v>0</v>
       </c>
       <c r="F75" t="n">
-        <v>51660.12</v>
+        <v>0</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
+          <t>1inch — re-routed executor-owned Referral(4011) in the unified stream.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>9998</t>
+          <t>4012</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -27441,7 +27805,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>10000</t>
+          <t>9001</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -27450,27 +27814,27 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>373.74</v>
+        <v>17730.23</v>
       </c>
       <c r="D77" t="n">
-        <v>547.46</v>
+        <v>14347.44</v>
       </c>
       <c r="E77" t="n">
-        <v>1161.68</v>
+        <v>19582.45</v>
       </c>
       <c r="F77" t="n">
-        <v>2082.88</v>
+        <v>51660.12</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+          <t>Synthetic code: USDS in Aave aEthUSDS; entire contract balance. Intraday TWA (clean methodology) — the deployed Dune query used EOD snapshots, which under-count ~20% on heavy-flow months.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10001</t>
+          <t>9998</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -27479,47 +27843,101 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>77410.08</v>
+        <v>0</v>
       </c>
       <c r="D78" t="n">
-        <v>64106.05</v>
+        <v>0</v>
       </c>
       <c r="E78" t="n">
-        <v>68681.05</v>
+        <v>0</v>
       </c>
       <c r="F78" t="n">
-        <v>210197.18</v>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>soter only</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>373.74</v>
+      </c>
+      <c r="D79" t="n">
+        <v>547.46</v>
+      </c>
+      <c r="E79" t="n">
+        <v>1161.68</v>
+      </c>
+      <c r="F79" t="n">
+        <v>2082.88</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Synthetic code: L2 sUSDS default PSM3 code 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>soter only</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>77410.08</v>
+      </c>
+      <c r="D80" t="n">
+        <v>64106.05</v>
+      </c>
+      <c r="E80" t="n">
+        <v>68681.05</v>
+      </c>
+      <c r="F80" t="n">
+        <v>210197.18</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Synthetic code: Smart-contract-held L2 sUSDS (code 0 split).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
           <t>13425</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>soter only</t>
         </is>
       </c>
-      <c r="C79" t="n">
+      <c r="C81" t="n">
         <v>858.01</v>
       </c>
-      <c r="D79" t="n">
+      <c r="D81" t="n">
         <v>774.97</v>
       </c>
-      <c r="E79" t="n">
+      <c r="E81" t="n">
         <v>858.01</v>
       </c>
-      <c r="F79" t="n">
+      <c r="F81" t="n">
         <v>2490.99</v>
       </c>
-      <c r="G79" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Restrict Skybase rewards to 2026
</commit_message>
<xml_diff>
--- a/hypersync-results/dr_comparison_hypersync.xlsx
+++ b/hypersync-results/dr_comparison_hypersync.xlsx
@@ -17511,51 +17511,21 @@
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
-      <c r="D127" t="n">
-        <v>300.81</v>
-      </c>
-      <c r="E127" t="n">
-        <v>197.7</v>
-      </c>
-      <c r="F127" t="n">
-        <v>156.26</v>
-      </c>
-      <c r="G127" t="n">
-        <v>154.44</v>
-      </c>
-      <c r="H127" t="n">
-        <v>149.32</v>
-      </c>
-      <c r="I127" t="n">
-        <v>138.39</v>
-      </c>
-      <c r="J127" t="n">
-        <v>16.73</v>
-      </c>
-      <c r="K127" t="n">
-        <v>10.02</v>
-      </c>
-      <c r="L127" t="n">
-        <v>8.970000000000001</v>
-      </c>
-      <c r="M127" t="n">
-        <v>8.91</v>
-      </c>
-      <c r="N127" t="n">
-        <v>8.94</v>
-      </c>
-      <c r="O127" t="n">
-        <v>4.38</v>
-      </c>
-      <c r="P127" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="Q127" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="R127" t="n">
-        <v>0.33</v>
-      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+      <c r="K127" t="inlineStr"/>
+      <c r="L127" t="inlineStr"/>
+      <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr"/>
+      <c r="O127" t="inlineStr"/>
+      <c r="P127" t="inlineStr"/>
+      <c r="Q127" t="inlineStr"/>
+      <c r="R127" t="inlineStr"/>
       <c r="S127" t="n">
         <v>0.33</v>
       </c>
@@ -17581,7 +17551,7 @@
         <v>12492.55</v>
       </c>
       <c r="AA127" t="n">
-        <v>28896.09</v>
+        <v>27740.24</v>
       </c>
       <c r="AB127" t="inlineStr">
         <is>
@@ -21169,7 +21139,7 @@
         <v>27740.24</v>
       </c>
       <c r="M42" t="n">
-        <v>1155.86</v>
+        <v>0</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -22170,7 +22140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22203,7 +22173,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -22215,37 +22185,37 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>300.8080383671237</v>
+        <v>0.3318514472871808</v>
       </c>
       <c r="E2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2026-01</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1997</v>
+        <v>1999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_risk_capital</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>197.7048212854454</v>
+        <v>177.6857204469182</v>
       </c>
       <c r="E3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -22257,58 +22227,58 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>156.2640116915537</v>
+        <v>0.3329049989406912</v>
       </c>
       <c r="E4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_flagship</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>154.4372667803067</v>
+        <v>8.620555888252163e-05</v>
       </c>
       <c r="E5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2026-02</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1997</v>
+        <v>1999</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_risk_capital</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>149.3197237671313</v>
+        <v>307.7580186696092</v>
       </c>
       <c r="E6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -22320,58 +22290,58 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>138.3937724247048</v>
+        <v>0.3339434963263763</v>
       </c>
       <c r="E7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_flagship</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>16.72518800773313</v>
+        <v>5425.078324149193</v>
       </c>
       <c r="E8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2026-03</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1997</v>
+        <v>1999</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_risk_capital</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10.02323501821356</v>
+        <v>147.2736416787795</v>
       </c>
       <c r="E9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -22383,58 +22353,58 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8.967148419076839</v>
+        <v>0.3349734848324279</v>
       </c>
       <c r="E10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_flagship</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>8.912793568136445</v>
+        <v>6454.40020769498</v>
       </c>
       <c r="E11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>2026-04</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1997</v>
+        <v>1999</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_risk_capital</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>8.937364988654359</v>
+        <v>26.59639852146469</v>
       </c>
       <c r="E12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -22446,58 +22416,58 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4.376165615994683</v>
+        <v>1.514372319701787</v>
       </c>
       <c r="E13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-10</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_flagship</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.3286696536304232</v>
+        <v>7020.719853450289</v>
       </c>
       <c r="E14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-11</t>
+          <t>2026-05</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1997</v>
+        <v>1999</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_risk_capital</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.3295678089045515</v>
+        <v>30.34189158796749</v>
       </c>
       <c r="E15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-12</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -22509,28 +22479,28 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.330739718172114</v>
+        <v>6953.518137125108</v>
       </c>
       <c r="E16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1997</v>
+        <v>1998</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>skybase_pendle</t>
+          <t>skybase_flagship</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.3318514472871808</v>
+        <v>4810.914277181574</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
@@ -22539,7 +22509,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -22551,7 +22521,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>177.6857204469182</v>
+        <v>20.23617948770795</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -22560,7 +22530,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -22572,7 +22542,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.3329049989406912</v>
+        <v>8291.323682686629</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
@@ -22581,7 +22551,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -22593,7 +22563,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>8.620555888252163e-05</v>
+        <v>4923.134510263595</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
@@ -22602,7 +22572,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -22614,7 +22584,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>307.7580186696092</v>
+        <v>21.14386762725331</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
@@ -22623,7 +22593,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -22635,7 +22605,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.3339434963263763</v>
+        <v>12492.54544984775</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
@@ -22644,7 +22614,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -22656,7 +22626,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>5425.078324149193</v>
+        <v>5594.92538693962</v>
       </c>
       <c r="E23" t="b">
         <v>1</v>
@@ -22665,7 +22635,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-03</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -22677,324 +22647,9 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>147.2736416787795</v>
+        <v>27.71695008796137</v>
       </c>
       <c r="E24" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1997</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>skybase_pendle</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>0.3349734848324279</v>
-      </c>
-      <c r="E25" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>1998</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>skybase_flagship</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>6454.40020769498</v>
-      </c>
-      <c r="E26" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>1999</v>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>skybase_risk_capital</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>26.59639852146469</v>
-      </c>
-      <c r="E27" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>1997</v>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>skybase_pendle</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>1.514372319701787</v>
-      </c>
-      <c r="E28" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>1998</v>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>skybase_flagship</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>7020.719853450289</v>
-      </c>
-      <c r="E29" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1999</v>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>skybase_risk_capital</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>30.34189158796749</v>
-      </c>
-      <c r="E30" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1997</v>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>skybase_pendle</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>6953.518137125108</v>
-      </c>
-      <c r="E31" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>1998</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>skybase_flagship</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>4810.914277181574</v>
-      </c>
-      <c r="E32" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>1999</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>skybase_risk_capital</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>20.23617948770795</v>
-      </c>
-      <c r="E33" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>1997</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>skybase_pendle</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>8291.323682686629</v>
-      </c>
-      <c r="E34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>1998</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>skybase_flagship</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>4923.134510263595</v>
-      </c>
-      <c r="E35" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>1999</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>skybase_risk_capital</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>21.14386762725331</v>
-      </c>
-      <c r="E36" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>1997</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>skybase_pendle</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>12492.54544984775</v>
-      </c>
-      <c r="E37" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>1998</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>skybase_flagship</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>5594.92538693962</v>
-      </c>
-      <c r="E38" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1999</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>skybase_risk_capital</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>27.71695008796137</v>
-      </c>
-      <c r="E39" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>